<commit_message>
agrego requirements.txt, grafico de promedio de ocio y path general
</commit_message>
<xml_diff>
--- a/output/analisis_sensibilidad.xlsx
+++ b/output/analisis_sensibilidad.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resumen Comparativo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Detalle por Escenario" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Datos Gráficos" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gráficos" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen Comparativo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle por Escenario" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos Gráficos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gráficos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -377,14 +377,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -408,7 +408,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -432,7 +432,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -484,14 +484,14 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -515,7 +515,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -539,7 +539,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -591,14 +591,14 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -622,7 +622,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -646,7 +646,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -697,8 +697,115 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Ociosidad Prom por Cargador (%)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Datos Gráficos'!B25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Datos Gráficos'!$A$26:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Datos Gráficos'!$B$26:$B$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Datos Gráficos'!C25</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Datos Gráficos'!$A$26:$A$28</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Datos Gráficos'!$C$26:$C$28</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -713,9 +820,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -735,9 +842,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -757,9 +864,31 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="4" name="Chart 4"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1080,7 +1209,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Simulación de 1440 minutos | Seed: 42 | 2026-04-26</t>
+          <t>Simulación de 1440 minutos | Seed: 42 | 2026-04-27</t>
         </is>
       </c>
     </row>
@@ -2006,7 +2135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2210,12 +2339,76 @@
         <v>89.70605342878281</v>
       </c>
     </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="36" t="inlineStr">
+        <is>
+          <t>Ociosidad Prom por Cargador (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Escenario</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>CSR</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="25" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="n">
+        <v>0.3881305269837859</v>
+      </c>
+      <c r="C26" s="21" t="n">
+        <v>0.6433803156961898</v>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="25" t="inlineStr">
+        <is>
+          <t>Eficiente</t>
+        </is>
+      </c>
+      <c r="B27" s="21" t="n">
+        <v>0.2747546389858979</v>
+      </c>
+      <c r="C27" s="21" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="16" customHeight="1">
+      <c r="A28" s="25" t="inlineStr">
+        <is>
+          <t>No eficiente</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="n">
+        <v>0.7659794279569117</v>
+      </c>
+      <c r="C28" s="21" t="n">
+        <v>0.6885206478167263</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A17:G17"/>
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A17:G17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualizamos arrepentimiento, formula eficiencia y formato excel
</commit_message>
<xml_diff>
--- a/output/analisis_sensibilidad.xlsx
+++ b/output/analisis_sensibilidad.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="33">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,17 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00F4D03F"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
@@ -64,17 +75,7 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
       <color rgb="00CA6F1E"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00C0392B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -91,12 +92,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="001E8449"/>
       <sz val="10"/>
     </font>
@@ -108,13 +103,8 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00F4D03F"/>
+      <color rgb="00AAAAAA"/>
       <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00888888"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -148,12 +138,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="001E8449"/>
       <sz val="18"/>
     </font>
@@ -229,8 +213,13 @@
       <color rgb="00C0392B"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -254,6 +243,46 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00163D64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000A2A47"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001B5E8A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A6EA0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A6636"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E7A3E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B2400"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008C2900"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00F2F3F4"/>
       </patternFill>
     </fill>
@@ -269,12 +298,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FDEBD0"/>
+        <fgColor rgb="00117A65"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FADBD8"/>
+        <fgColor rgb="00FDEBD0"/>
       </patternFill>
     </fill>
     <fill>
@@ -309,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="64">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -318,182 +347,212 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="8" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="9" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="19" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="21" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="20" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="20" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="17" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="18" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="26" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="28" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="31" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="31" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="28" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="32" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -890,7 +949,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Score de Eficiencia (↓ mejor)</a:t>
+              <a:t>Score de Eficiencia (↑ mayor = mejor)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -949,6 +1008,135 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="10"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>% Abandono por Escenario: CR vs CSR</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Eficiencia'!B17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="2E86C1"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Eficiencia'!$A$18:$A$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Eficiencia'!$B$18:$B$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Eficiencia'!C17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:solidFill>
+              <a:srgbClr val="117A65"/>
+            </a:solidFill>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Eficiencia'!$A$18:$A$20</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Eficiencia'!$C$18:$C$20</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Tasa de abandono</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0%" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -1053,6 +1241,28 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>5</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="3600000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1350,7 +1560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1375,388 +1585,398 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  100 réplicas  ·  43200 min c/u  ·  Seed: aleatorio  ·  Generado: 28/04/2026 16:16</t>
+          <t xml:space="preserve">  100 réplicas  ·  1440 min c/u  ·  Seed: aleatorio  ·  Generado: 28/04/2026 16:48</t>
         </is>
       </c>
     </row>
     <row r="3" ht="4" customHeight="1">
       <c r="A3" s="3" t="n"/>
     </row>
-    <row r="4" ht="38" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>Eficiente</t>
+        </is>
+      </c>
+      <c r="G4" s="7" t="inlineStr">
+        <is>
+          <t>No eficiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Métrica</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Unidad</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Real
-CR</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Real
-CSR</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Eficiente
-CR</t>
-        </is>
-      </c>
-      <c r="F4" s="4" t="inlineStr">
-        <is>
-          <t>Eficiente
-CSR</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>No efic.
-CR</t>
-        </is>
-      </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>No efic.
-CSR</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>CSR</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>CSR</t>
+        </is>
+      </c>
+      <c r="G5" s="13" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="H5" s="14" t="inlineStr">
+        <is>
+          <t>CSR</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="3" customHeight="1">
+      <c r="A6" s="3" t="n"/>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="3" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>N° Cargadores</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C7" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D7" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E7" s="17" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H5" s="7" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="G7" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
         <is>
           <t>Llegadas promedio</t>
         </is>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B8" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C6" s="10" t="n">
-        <v>890.36</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>310.28</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>1202.71</v>
-      </c>
-      <c r="F6" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G6" s="10" t="n">
-        <v>887.34</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>311.66</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="C8" s="20" t="n">
+        <v>30.28</v>
+      </c>
+      <c r="D8" s="20" t="n">
+        <v>10.61</v>
+      </c>
+      <c r="E8" s="20" t="n">
+        <v>30.61</v>
+      </c>
+      <c r="F8" s="20" t="n">
+        <v>10.04</v>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t>Atendidos promedio</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C7" s="12" t="n">
-        <v>773.96</v>
-      </c>
-      <c r="D7" s="12" t="n">
-        <v>249.78</v>
-      </c>
-      <c r="E7" s="12" t="n">
-        <v>960.48</v>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G7" s="12" t="n">
-        <v>882.8</v>
-      </c>
-      <c r="H7" s="12" t="n">
-        <v>304.94</v>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="C9" s="21" t="n">
+        <v>26.36</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>8.58</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>30.46</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>8.279999999999999</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>10.4</v>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="18" t="inlineStr">
         <is>
           <t>Arrepentidos prom.</t>
         </is>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B10" s="19" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="C8" s="10" t="n">
-        <v>116.4</v>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>242.23</v>
-      </c>
-      <c r="F8" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G8" s="10" t="n">
-        <v>4.54</v>
-      </c>
-      <c r="H8" s="10" t="n">
-        <v>6.72</v>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="C10" s="20" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="D10" s="20" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="E10" s="20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>% Abandono</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C9" s="13" t="n">
-        <v>0.1305903779074988</v>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>0.1945252402134508</v>
-      </c>
-      <c r="E9" s="14" t="n">
-        <v>0.2012924677053878</v>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G9" s="15" t="n">
-        <v>0.005102422455934052</v>
-      </c>
-      <c r="H9" s="15" t="n">
-        <v>0.02146389462993271</v>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="C11" s="22" t="n">
+        <v>0.1253394588482308</v>
+      </c>
+      <c r="D11" s="22" t="n">
+        <v>0.1796217663055898</v>
+      </c>
+      <c r="E11" s="23" t="n">
+        <v>0.004607572894210825</v>
+      </c>
+      <c r="F11" s="22" t="n">
+        <v>0.1583791581655359</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="18" t="inlineStr">
         <is>
           <t>Espera promedio</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
+      <c r="B12" s="19" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="C10" s="16" t="n">
-        <v>6.723103590118701</v>
-      </c>
-      <c r="D10" s="16" t="n">
-        <v>10.06956692321773</v>
-      </c>
-      <c r="E10" s="16" t="n">
-        <v>10.56808631075325</v>
-      </c>
-      <c r="F10" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G10" s="16" t="n">
-        <v>0.362153191219949</v>
-      </c>
-      <c r="H10" s="16" t="n">
-        <v>0.8817627410142286</v>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="C12" s="24" t="n">
+        <v>5.761531231455991</v>
+      </c>
+      <c r="D12" s="24" t="n">
+        <v>9.597721506031091</v>
+      </c>
+      <c r="E12" s="24" t="n">
+        <v>0.3818516294810471</v>
+      </c>
+      <c r="F12" s="24" t="n">
+        <v>7.314134129313196</v>
+      </c>
+      <c r="G12" s="24" t="n">
+        <v>0.01202859565170951</v>
+      </c>
+      <c r="H12" s="24" t="n">
+        <v>0.006482986361158964</v>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Tiempo en sistema</t>
         </is>
       </c>
-      <c r="B11" s="6" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>min</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n">
-        <v>42.44198717348761</v>
-      </c>
-      <c r="D11" s="17" t="n">
-        <v>91.09072609553201</v>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>46.66642213672038</v>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G11" s="17" t="n">
-        <v>35.43044686499417</v>
-      </c>
-      <c r="H11" s="17" t="n">
-        <v>80.57939164804974</v>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="C13" s="25" t="n">
+        <v>41.43013127298266</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>89.40976115474801</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>35.3245359283821</v>
+      </c>
+      <c r="F13" s="25" t="n">
+        <v>87.80994943672478</v>
+      </c>
+      <c r="G13" s="25" t="n">
+        <v>35.12663786201732</v>
+      </c>
+      <c r="H13" s="25" t="n">
+        <v>80.03624894523395</v>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="18" t="inlineStr">
         <is>
           <t>Ociosidad cargadores</t>
         </is>
       </c>
-      <c r="B12" s="9" t="inlineStr">
+      <c r="B14" s="19" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
-        <v>0.3603615649540284</v>
-      </c>
-      <c r="D12" s="18" t="n">
-        <v>0.5318789455758461</v>
-      </c>
-      <c r="E12" s="18" t="n">
-        <v>0.197877863479211</v>
-      </c>
-      <c r="F12" s="11" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="G12" s="18" t="n">
-        <v>0.6417266500063495</v>
-      </c>
-      <c r="H12" s="18" t="n">
-        <v>0.7188206690342753</v>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="C14" s="26" t="n">
+        <v>0.3541506500866051</v>
+      </c>
+      <c r="D14" s="26" t="n">
+        <v>0.5329493198082061</v>
+      </c>
+      <c r="E14" s="26" t="n">
+        <v>0.6318567550864226</v>
+      </c>
+      <c r="F14" s="26" t="n">
+        <v>0.5471170794734832</v>
+      </c>
+      <c r="G14" s="26" t="n">
+        <v>0.7596752161205959</v>
+      </c>
+      <c r="H14" s="26" t="n">
+        <v>0.8565395884989202</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
         <is>
           <t>Abandono total</t>
         </is>
       </c>
-      <c r="B13" s="20" t="inlineStr">
+      <c r="B15" s="28" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C13" s="21" t="n">
-        <v>0.1473380863539446</v>
-      </c>
-      <c r="D13" s="21" t="n">
-        <v>0.1473380863539446</v>
-      </c>
-      <c r="E13" s="22" t="n">
-        <v>0.2014034971023771</v>
-      </c>
-      <c r="F13" s="22" t="n">
-        <v>0.2014034971023771</v>
-      </c>
-      <c r="G13" s="23" t="n">
-        <v>0.009391159299416181</v>
-      </c>
-      <c r="H13" s="23" t="n">
-        <v>0.009391159299416181</v>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="24" t="inlineStr">
-        <is>
-          <t>Eficiencia global (↓ mejor)</t>
-        </is>
-      </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="C15" s="29" t="n">
+        <v>0.1455123502078748</v>
+      </c>
+      <c r="D15" s="29" t="n">
+        <v>0.1455123502078748</v>
+      </c>
+      <c r="E15" s="30" t="n">
+        <v>0.04698646986469865</v>
+      </c>
+      <c r="F15" s="30" t="n">
+        <v>0.04698646986469865</v>
+      </c>
+      <c r="G15" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>Eficiencia global (⭡ mayor = mejor)</t>
+        </is>
+      </c>
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="C14" s="26" t="n">
-        <v>-21.66272822547933</v>
-      </c>
-      <c r="D14" s="27" t="inlineStr">
+      <c r="C16" s="33" t="n">
+        <v>0.2782250075262972</v>
+      </c>
+      <c r="D16" s="34" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="26" t="n">
-        <v>-9.393893173960548</v>
-      </c>
-      <c r="F14" s="27" t="inlineStr">
+      <c r="E16" s="33" t="n">
+        <v>0.55920114252168</v>
+      </c>
+      <c r="F16" s="34" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G14" s="26" t="n">
-        <v>-33.03712892316468</v>
-      </c>
-      <c r="H14" s="27" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="G16" s="35" t="n">
+        <v>0.5916969534265795</v>
+      </c>
+      <c r="H16" s="32" t="inlineStr">
+        <is>
+          <t>★ MEJOR</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="6">
+    <mergeCell ref="G4:H4"/>
     <mergeCell ref="A1:J1"/>
+    <mergeCell ref="E4:F4"/>
     <mergeCell ref="A3:J3"/>
     <mergeCell ref="A2:J2"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1780,179 +2000,179 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>PANEL DE KPIs POR ESCENARIO</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="29" t="inlineStr">
+      <c r="A2" s="37" t="inlineStr">
         <is>
           <t>Comparación rápida entre escenarios simulados</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="38" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="38" t="inlineStr">
         <is>
           <t>Eficiente</t>
         </is>
       </c>
-      <c r="E4" s="30" t="inlineStr">
-        <is>
-          <t>No eficiente</t>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>No eficiente ★</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="31" t="inlineStr">
+      <c r="A5" s="40" t="inlineStr">
         <is>
           <t>Abandono total</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="40" t="inlineStr">
         <is>
           <t>Abandono total</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="40" t="inlineStr">
         <is>
           <t>Abandono total</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="32" t="n">
-        <v>0.1305903779074988</v>
-      </c>
-      <c r="C6" s="33" t="n">
-        <v>0.2012924677053878</v>
-      </c>
-      <c r="E6" s="34" t="n">
-        <v>0.005102422455934052</v>
+      <c r="A6" s="41" t="n">
+        <v>0.1253394588482308</v>
+      </c>
+      <c r="C6" s="42" t="n">
+        <v>0.004607572894210825</v>
+      </c>
+      <c r="E6" s="42" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="7" ht="5" customHeight="1">
-      <c r="A7" s="35" t="n"/>
-      <c r="B7" s="35" t="n"/>
-      <c r="C7" s="35" t="n"/>
-      <c r="D7" s="35" t="n"/>
-      <c r="E7" s="35" t="n"/>
-      <c r="F7" s="35" t="n"/>
+      <c r="A7" s="43" t="n"/>
+      <c r="B7" s="43" t="n"/>
+      <c r="C7" s="43" t="n"/>
+      <c r="D7" s="43" t="n"/>
+      <c r="E7" s="43" t="n"/>
+      <c r="F7" s="43" t="n"/>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="31" t="inlineStr">
+      <c r="A8" s="40" t="inlineStr">
         <is>
           <t>Espera prom. CR</t>
         </is>
       </c>
-      <c r="C8" s="31" t="inlineStr">
+      <c r="C8" s="40" t="inlineStr">
         <is>
           <t>Espera prom. CR</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="40" t="inlineStr">
         <is>
           <t>Espera prom. CR</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="36" t="n">
-        <v>6.723103590118701</v>
-      </c>
-      <c r="C9" s="36" t="n">
-        <v>10.56808631075325</v>
-      </c>
-      <c r="E9" s="36" t="n">
-        <v>0.362153191219949</v>
+      <c r="A9" s="44" t="n">
+        <v>5.761531231455991</v>
+      </c>
+      <c r="C9" s="44" t="n">
+        <v>0.3818516294810471</v>
+      </c>
+      <c r="E9" s="44" t="n">
+        <v>0.01202859565170951</v>
       </c>
     </row>
     <row r="10" ht="5" customHeight="1">
-      <c r="A10" s="35" t="n"/>
-      <c r="B10" s="35" t="n"/>
-      <c r="C10" s="35" t="n"/>
-      <c r="D10" s="35" t="n"/>
-      <c r="E10" s="35" t="n"/>
-      <c r="F10" s="35" t="n"/>
+      <c r="A10" s="43" t="n"/>
+      <c r="B10" s="43" t="n"/>
+      <c r="C10" s="43" t="n"/>
+      <c r="D10" s="43" t="n"/>
+      <c r="E10" s="43" t="n"/>
+      <c r="F10" s="43" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="31" t="inlineStr">
+      <c r="A11" s="40" t="inlineStr">
         <is>
           <t>Ociosidad CR</t>
         </is>
       </c>
-      <c r="C11" s="31" t="inlineStr">
+      <c r="C11" s="40" t="inlineStr">
         <is>
           <t>Ociosidad CR</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="40" t="inlineStr">
         <is>
           <t>Ociosidad CR</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="37" t="n">
-        <v>0.3603615649540284</v>
-      </c>
-      <c r="C12" s="37" t="n">
-        <v>0.197877863479211</v>
-      </c>
-      <c r="E12" s="37" t="n">
-        <v>0.6417266500063495</v>
+      <c r="A12" s="45" t="n">
+        <v>0.3541506500866051</v>
+      </c>
+      <c r="C12" s="45" t="n">
+        <v>0.6318567550864226</v>
+      </c>
+      <c r="E12" s="45" t="n">
+        <v>0.7596752161205959</v>
       </c>
     </row>
     <row r="13" ht="5" customHeight="1">
-      <c r="A13" s="35" t="n"/>
-      <c r="B13" s="35" t="n"/>
-      <c r="C13" s="35" t="n"/>
-      <c r="D13" s="35" t="n"/>
-      <c r="E13" s="35" t="n"/>
-      <c r="F13" s="35" t="n"/>
+      <c r="A13" s="43" t="n"/>
+      <c r="B13" s="43" t="n"/>
+      <c r="C13" s="43" t="n"/>
+      <c r="D13" s="43" t="n"/>
+      <c r="E13" s="43" t="n"/>
+      <c r="F13" s="43" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="31" t="inlineStr">
+      <c r="A14" s="40" t="inlineStr">
         <is>
           <t>Atendidos CR</t>
         </is>
       </c>
-      <c r="C14" s="31" t="inlineStr">
+      <c r="C14" s="40" t="inlineStr">
         <is>
           <t>Atendidos CR</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="E14" s="40" t="inlineStr">
         <is>
           <t>Atendidos CR</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="38" t="n">
-        <v>773.96</v>
-      </c>
-      <c r="C15" s="38" t="n">
-        <v>960.48</v>
-      </c>
-      <c r="E15" s="38" t="n">
-        <v>882.8</v>
+      <c r="A15" s="46" t="n">
+        <v>26.36</v>
+      </c>
+      <c r="C15" s="46" t="n">
+        <v>30.46</v>
+      </c>
+      <c r="E15" s="46" t="n">
+        <v>29.7</v>
       </c>
     </row>
     <row r="16" ht="5" customHeight="1">
-      <c r="A16" s="35" t="n"/>
-      <c r="B16" s="35" t="n"/>
-      <c r="C16" s="35" t="n"/>
-      <c r="D16" s="35" t="n"/>
-      <c r="E16" s="35" t="n"/>
-      <c r="F16" s="35" t="n"/>
+      <c r="A16" s="43" t="n"/>
+      <c r="B16" s="43" t="n"/>
+      <c r="C16" s="43" t="n"/>
+      <c r="D16" s="43" t="n"/>
+      <c r="E16" s="43" t="n"/>
+      <c r="F16" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="29">
@@ -2007,229 +2227,229 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>INSIGHTS AUTOMÁTICOS</t>
         </is>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1">
-      <c r="A3" s="39" t="inlineStr">
+      <c r="A3" s="47" t="inlineStr">
         <is>
           <t>📊  Escenario: Real</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Abandono total:</t>
         </is>
       </c>
-      <c r="B4" s="40" t="inlineStr">
-        <is>
-          <t>14.7%</t>
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>14.6%</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Atendidos CR / CSR:</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>774 / 250</t>
+      <c r="B5" s="49" t="inlineStr">
+        <is>
+          <t>26 / 9</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Espera prom. CR:</t>
         </is>
       </c>
-      <c r="B6" s="42" t="inlineStr">
-        <is>
-          <t>6.7 min</t>
+      <c r="B6" s="50" t="inlineStr">
+        <is>
+          <t>5.8 min</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Espera prom. CSR:</t>
         </is>
       </c>
-      <c r="B7" s="42" t="inlineStr">
-        <is>
-          <t>10.1 min</t>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>9.6 min</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Eficiencia global:</t>
         </is>
       </c>
-      <c r="B8" s="43" t="inlineStr">
-        <is>
-          <t>-21.663</t>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>0.278  (↑ mayor = mejor)</t>
         </is>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="44" t="inlineStr">
+      <c r="A9" s="52" t="inlineStr">
         <is>
           <t>⚡  Pérdida moderada — monitorear horas pico.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="47" t="inlineStr">
         <is>
           <t>📊  Escenario: Eficiente</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Abandono total:</t>
         </is>
       </c>
-      <c r="B12" s="45" t="inlineStr">
-        <is>
-          <t>20.1%</t>
+      <c r="B12" s="53" t="inlineStr">
+        <is>
+          <t>4.7%</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Atendidos CR / CSR:</t>
         </is>
       </c>
-      <c r="B13" s="41" t="inlineStr">
-        <is>
-          <t>960 / 0</t>
+      <c r="B13" s="49" t="inlineStr">
+        <is>
+          <t>30 / 8</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Espera prom. CR:</t>
         </is>
       </c>
-      <c r="B14" s="42" t="inlineStr">
-        <is>
-          <t>10.6 min</t>
+      <c r="B14" s="50" t="inlineStr">
+        <is>
+          <t>0.4 min</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Espera prom. CSR:</t>
         </is>
       </c>
-      <c r="B15" s="42" t="inlineStr">
+      <c r="B15" s="50" t="inlineStr">
+        <is>
+          <t>7.3 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Eficiencia global:</t>
+        </is>
+      </c>
+      <c r="B16" s="51" t="inlineStr">
+        <is>
+          <t>0.559  (↑ mayor = mejor)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="54" t="inlineStr">
+        <is>
+          <t>✅  Sistema eficiente — demanda bien gestionada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="47" t="inlineStr">
+        <is>
+          <t>📊  Escenario: No eficiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>Abandono total:</t>
+        </is>
+      </c>
+      <c r="B20" s="53" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>Atendidos CR / CSR:</t>
+        </is>
+      </c>
+      <c r="B21" s="49" t="inlineStr">
+        <is>
+          <t>30 / 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Espera prom. CR:</t>
+        </is>
+      </c>
+      <c r="B22" s="50" t="inlineStr">
         <is>
           <t>0.0 min</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>Espera prom. CSR:</t>
+        </is>
+      </c>
+      <c r="B23" s="50" t="inlineStr">
+        <is>
+          <t>0.0 min</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>Eficiencia global:</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
-        <is>
-          <t>-9.394</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="46" t="inlineStr">
-        <is>
-          <t>⚠️  Alta pérdida de demanda — considerar más cargadores.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="39" t="inlineStr">
-        <is>
-          <t>📊  Escenario: No eficiente</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>Abandono total:</t>
-        </is>
-      </c>
-      <c r="B20" s="47" t="inlineStr">
-        <is>
-          <t>0.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Atendidos CR / CSR:</t>
-        </is>
-      </c>
-      <c r="B21" s="41" t="inlineStr">
-        <is>
-          <t>883 / 305</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Espera prom. CR:</t>
-        </is>
-      </c>
-      <c r="B22" s="42" t="inlineStr">
-        <is>
-          <t>0.4 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Espera prom. CSR:</t>
-        </is>
-      </c>
-      <c r="B23" s="42" t="inlineStr">
-        <is>
-          <t>0.9 min</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>Eficiencia global:</t>
-        </is>
-      </c>
-      <c r="B24" s="43" t="inlineStr">
-        <is>
-          <t>-33.037</t>
+      <c r="B24" s="51" t="inlineStr">
+        <is>
+          <t>0.592  (↑ mayor = mejor)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="48" t="inlineStr">
+      <c r="A25" s="54" t="inlineStr">
         <is>
           <t>✅  Sistema eficiente — demanda bien gestionada.</t>
         </is>
@@ -2282,94 +2502,94 @@
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>GRÁFICOS COMPARATIVOS</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="49" t="inlineStr">
+      <c r="A3" s="55" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="B3" s="49" t="inlineStr">
+      <c r="B3" s="55" t="inlineStr">
         <is>
           <t>% Abandono CR</t>
         </is>
       </c>
-      <c r="C3" s="49" t="inlineStr">
+      <c r="C3" s="55" t="inlineStr">
         <is>
           <t>Espera CR (min)</t>
         </is>
       </c>
-      <c r="D3" s="49" t="inlineStr">
+      <c r="D3" s="55" t="inlineStr">
         <is>
           <t>Ociosidad CR (%)</t>
         </is>
       </c>
-      <c r="E3" s="49" t="inlineStr">
+      <c r="E3" s="55" t="inlineStr">
         <is>
           <t>Atendidos CR</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="B4" s="50" t="n">
-        <v>0.1305903779074988</v>
-      </c>
-      <c r="C4" s="17" t="n">
-        <v>6.723103590118701</v>
-      </c>
-      <c r="D4" s="50" t="n">
-        <v>0.3603615649540284</v>
-      </c>
-      <c r="E4" s="12" t="n">
-        <v>773.96</v>
+      <c r="B4" s="56" t="n">
+        <v>0.1253394588482308</v>
+      </c>
+      <c r="C4" s="25" t="n">
+        <v>5.761531231455991</v>
+      </c>
+      <c r="D4" s="56" t="n">
+        <v>0.3541506500866051</v>
+      </c>
+      <c r="E4" s="21" t="n">
+        <v>26.36</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="57" t="inlineStr">
         <is>
           <t>Eficiente</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
-        <v>0.2012924677053878</v>
-      </c>
-      <c r="C5" s="16" t="n">
-        <v>10.56808631075325</v>
-      </c>
-      <c r="D5" s="18" t="n">
-        <v>0.197877863479211</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <v>960.48</v>
+      <c r="B5" s="26" t="n">
+        <v>0.004607572894210825</v>
+      </c>
+      <c r="C5" s="24" t="n">
+        <v>0.3818516294810471</v>
+      </c>
+      <c r="D5" s="26" t="n">
+        <v>0.6318567550864226</v>
+      </c>
+      <c r="E5" s="20" t="n">
+        <v>30.46</v>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>No eficiente</t>
         </is>
       </c>
-      <c r="B6" s="50" t="n">
-        <v>0.005102422455934052</v>
-      </c>
-      <c r="C6" s="17" t="n">
-        <v>0.362153191219949</v>
-      </c>
-      <c r="D6" s="50" t="n">
-        <v>0.6417266500063495</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>882.8</v>
+      <c r="B6" s="56" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>0.01202859565170951</v>
+      </c>
+      <c r="D6" s="56" t="n">
+        <v>0.7596752161205959</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>29.7</v>
       </c>
     </row>
   </sheetData>
@@ -2387,106 +2607,107 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
-      <c r="A1" s="28" t="inlineStr">
+      <c r="A1" s="36" t="inlineStr">
         <is>
           <t>RANKING DE EFICIENCIA GLOBAL</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="51" t="inlineStr">
-        <is>
-          <t>Score compuesto: 0.4×Espera + 0.3×Ociosidad + 0.2×Abandono − 0.1×Atendidos  (↓ mejor)</t>
+      <c r="A2" s="58" t="inlineStr">
+        <is>
+          <t>Score compuesto (↑ mayor = mejor):  −0.4×Espera − 0.3×Ociosidad − 0.2×Abandono + 0.1×Atendidos</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Pos.</t>
         </is>
       </c>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="8" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="8" t="inlineStr">
         <is>
           <t>Evaluación</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="52" t="inlineStr">
+      <c r="A5" s="59" t="inlineStr">
         <is>
           <t>🥇 #1</t>
         </is>
       </c>
-      <c r="B5" s="53" t="inlineStr">
+      <c r="B5" s="60" t="inlineStr">
         <is>
           <t>No eficiente</t>
         </is>
       </c>
-      <c r="C5" s="54" t="n">
-        <v>-33.03712892316468</v>
-      </c>
-      <c r="D5" s="55" t="inlineStr">
+      <c r="C5" s="61" t="n">
+        <v>0.5916969534265795</v>
+      </c>
+      <c r="D5" s="62" t="inlineStr">
         <is>
           <t>Óptimo</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="56" t="inlineStr">
+      <c r="A6" s="63" t="inlineStr">
         <is>
           <t>🥈 #2</t>
         </is>
       </c>
-      <c r="B6" s="57" t="inlineStr">
+      <c r="B6" s="64" t="inlineStr">
+        <is>
+          <t>Eficiente</t>
+        </is>
+      </c>
+      <c r="C6" s="65" t="n">
+        <v>0.55920114252168</v>
+      </c>
+      <c r="D6" s="66" t="inlineStr">
+        <is>
+          <t>Aceptable</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="67" t="inlineStr">
+        <is>
+          <t>🥉 #3</t>
+        </is>
+      </c>
+      <c r="B7" s="68" t="inlineStr">
         <is>
           <t>Real</t>
         </is>
       </c>
-      <c r="C6" s="58" t="n">
-        <v>-21.66272822547933</v>
-      </c>
-      <c r="D6" s="59" t="inlineStr">
-        <is>
-          <t>Aceptable</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="60" t="inlineStr">
-        <is>
-          <t>🥉 #3</t>
-        </is>
-      </c>
-      <c r="B7" s="61" t="inlineStr">
-        <is>
-          <t>Eficiente</t>
-        </is>
-      </c>
-      <c r="C7" s="62" t="n">
-        <v>-9.393893173960548</v>
-      </c>
-      <c r="D7" s="63" t="inlineStr">
+      <c r="C7" s="69" t="n">
+        <v>0.2782250075262972</v>
+      </c>
+      <c r="D7" s="70" t="inlineStr">
         <is>
           <t>Mejorable</t>
         </is>
@@ -2511,33 +2732,97 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>-33.03712892316468</v>
+        <v>0.5916969534265795</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Real</t>
+          <t>Eficiente</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>-21.66272822547933</v>
+        <v>0.55920114252168</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2782250075262972</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="71" t="inlineStr">
+        <is>
+          <t>Comparación % abandono por tipo de cargador</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="55" t="inlineStr">
+        <is>
+          <t>Escenario</t>
+        </is>
+      </c>
+      <c r="B17" s="55" t="inlineStr">
+        <is>
+          <t>CR</t>
+        </is>
+      </c>
+      <c r="C17" s="55" t="inlineStr">
+        <is>
+          <t>CSR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="72" t="inlineStr">
+        <is>
+          <t>Real</t>
+        </is>
+      </c>
+      <c r="B18" s="73" t="n">
+        <v>0.1253394588482308</v>
+      </c>
+      <c r="C18" s="73" t="n">
+        <v>0.1796217663055898</v>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="72" t="inlineStr">
+        <is>
           <t>Eficiente</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>-9.393893173960548</v>
+      <c r="B19" s="73" t="n">
+        <v>0.004607572894210825</v>
+      </c>
+      <c r="C19" s="73" t="n">
+        <v>0.1583791581655359</v>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="72" t="inlineStr">
+        <is>
+          <t>No eficiente</t>
+        </is>
+      </c>
+      <c r="B20" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" s="73" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:D16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>